<commit_message>
data: MI355X MXFP4 EP=1 TP=4 profiling + breakdown (chat c=64)
Co-Authored-By: Claude Opus 4 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep1_tp4_rocm722_profiling/prefill_breakdown_c64.xlsx
+++ b/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep1_tp4_rocm722_profiling/prefill_breakdown_c64.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8.319000000000001</v>
+        <v>8.239000000000001</v>
       </c>
       <c r="D2" t="n">
         <v>0.7</v>
       </c>
       <c r="E2" t="n">
-        <v>339.7190000000001</v>
+        <v>348.199</v>
       </c>
       <c r="F2" t="n">
-        <v>30.3</v>
+        <v>30.7</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -492,10 +492,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>317.201</v>
+        <v>329.081</v>
       </c>
       <c r="D3" t="n">
-        <v>28.3</v>
+        <v>29</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
@@ -507,10 +507,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>14.199</v>
+        <v>10.879</v>
       </c>
       <c r="D4" t="n">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
@@ -527,13 +527,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.799</v>
+        <v>5.919</v>
       </c>
       <c r="D5" t="n">
         <v>0.5</v>
       </c>
       <c r="E5" t="n">
-        <v>24.278</v>
+        <v>25.038</v>
       </c>
       <c r="F5" t="n">
         <v>2.2</v>
@@ -548,10 +548,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18.479</v>
+        <v>19.119</v>
       </c>
       <c r="D6" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -568,16 +568,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>4.239</v>
+        <v>4.039</v>
       </c>
       <c r="D7" t="n">
         <v>0.4</v>
       </c>
       <c r="E7" t="n">
-        <v>360.234</v>
+        <v>369.954</v>
       </c>
       <c r="F7" t="n">
-        <v>32.2</v>
+        <v>32.6</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -589,10 +589,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5.039</v>
+        <v>5.239</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9.959</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D9" t="n">
         <v>0.9</v>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6.2</v>
+        <v>5.959</v>
       </c>
       <c r="D10" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7.399</v>
+        <v>7.439</v>
       </c>
       <c r="D11" t="n">
         <v>0.7</v>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>177.84</v>
+        <v>180.4</v>
       </c>
       <c r="D12" t="n">
         <v>15.9</v>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>4.199</v>
+        <v>4.039</v>
       </c>
       <c r="D14" t="n">
         <v>0.4</v>
@@ -694,10 +694,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>140.96</v>
+        <v>148.64</v>
       </c>
       <c r="D15" t="n">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
@@ -714,16 +714,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>347.202</v>
+        <v>342.882</v>
       </c>
       <c r="D16" t="n">
-        <v>31</v>
+        <v>30.2</v>
       </c>
       <c r="E16" t="n">
-        <v>360.361</v>
+        <v>355.201</v>
       </c>
       <c r="F16" t="n">
-        <v>32.2</v>
+        <v>31.3</v>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
@@ -735,10 +735,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>13.159</v>
+        <v>12.319</v>
       </c>
       <c r="D17" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
@@ -755,16 +755,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6.119</v>
+        <v>5.999</v>
       </c>
       <c r="D18" t="n">
         <v>0.5</v>
       </c>
       <c r="E18" t="n">
-        <v>35.718</v>
+        <v>35.318</v>
       </c>
       <c r="F18" t="n">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>29.599</v>
+        <v>29.319</v>
       </c>
       <c r="D19" t="n">
         <v>2.6</v>
@@ -792,7 +792,7 @@
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="n">
-        <v>1120.31</v>
+        <v>1133.71</v>
       </c>
       <c r="D20" t="n">
         <v>100</v>
@@ -872,10 +872,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>664.403</v>
+        <v>671.963</v>
       </c>
       <c r="D2" t="n">
-        <v>332.202</v>
+        <v>335.981</v>
       </c>
       <c r="E2" t="n">
         <v>59.3</v>
@@ -891,10 +891,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>177.84</v>
+        <v>180.4</v>
       </c>
       <c r="D3" t="n">
-        <v>177.84</v>
+        <v>180.4</v>
       </c>
       <c r="E3" t="n">
         <v>15.9</v>
@@ -910,13 +910,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>140.96</v>
+        <v>148.64</v>
       </c>
       <c r="D4" t="n">
-        <v>140.96</v>
+        <v>148.64</v>
       </c>
       <c r="E4" t="n">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="5">
@@ -929,10 +929,10 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>29.599</v>
+        <v>29.319</v>
       </c>
       <c r="D5" t="n">
-        <v>29.599</v>
+        <v>29.319</v>
       </c>
       <c r="E5" t="n">
         <v>2.6</v>
@@ -948,13 +948,13 @@
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>27.358</v>
+        <v>23.198</v>
       </c>
       <c r="D6" t="n">
-        <v>13.679</v>
+        <v>11.599</v>
       </c>
       <c r="E6" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -967,13 +967,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="n">
-        <v>18.479</v>
+        <v>19.119</v>
       </c>
       <c r="D7" t="n">
-        <v>18.479</v>
+        <v>19.119</v>
       </c>
       <c r="E7" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="8">
@@ -986,10 +986,10 @@
         <v>2</v>
       </c>
       <c r="C8" t="n">
-        <v>10.599</v>
+        <v>10.358</v>
       </c>
       <c r="D8" t="n">
-        <v>5.3</v>
+        <v>5.179</v>
       </c>
       <c r="E8" t="n">
         <v>0.9</v>
@@ -1005,10 +1005,10 @@
         <v>1</v>
       </c>
       <c r="C9" t="n">
-        <v>9.959</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="D9" t="n">
-        <v>9.959</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E9" t="n">
         <v>0.9</v>
@@ -1024,10 +1024,10 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>8.319000000000001</v>
+        <v>8.239000000000001</v>
       </c>
       <c r="D10" t="n">
-        <v>8.319000000000001</v>
+        <v>8.239000000000001</v>
       </c>
       <c r="E10" t="n">
         <v>0.7</v>
@@ -1043,10 +1043,10 @@
         <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>7.399</v>
+        <v>7.439</v>
       </c>
       <c r="D11" t="n">
-        <v>7.399</v>
+        <v>7.439</v>
       </c>
       <c r="E11" t="n">
         <v>0.7</v>
@@ -1062,10 +1062,10 @@
         <v>1</v>
       </c>
       <c r="C12" t="n">
-        <v>6.119</v>
+        <v>5.999</v>
       </c>
       <c r="D12" t="n">
-        <v>6.119</v>
+        <v>5.999</v>
       </c>
       <c r="E12" t="n">
         <v>0.5</v>
@@ -1081,10 +1081,10 @@
         <v>1</v>
       </c>
       <c r="C13" t="n">
-        <v>5.799</v>
+        <v>5.919</v>
       </c>
       <c r="D13" t="n">
-        <v>5.799</v>
+        <v>5.919</v>
       </c>
       <c r="E13" t="n">
         <v>0.5</v>
@@ -1100,13 +1100,13 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>5.039</v>
+        <v>5.239</v>
       </c>
       <c r="D14" t="n">
-        <v>5.039</v>
+        <v>5.239</v>
       </c>
       <c r="E14" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="15">
@@ -1119,10 +1119,10 @@
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>4.239</v>
+        <v>4.039</v>
       </c>
       <c r="D15" t="n">
-        <v>4.239</v>
+        <v>4.039</v>
       </c>
       <c r="E15" t="n">
         <v>0.4</v>
@@ -1138,10 +1138,10 @@
         <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>4.199</v>
+        <v>4.039</v>
       </c>
       <c r="D16" t="n">
-        <v>4.199</v>
+        <v>4.039</v>
       </c>
       <c r="E16" t="n">
         <v>0.4</v>

</xml_diff>